<commit_message>
Republish experimental thematic and framing analysis
</commit_message>
<xml_diff>
--- a/archive/histogram-themes-frames-2015-2025.xlsx
+++ b/archive/histogram-themes-frames-2015-2025.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Themes by Year'!$A$1:$K$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Frame Totals'!$A$1:$C$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Frames by Year'!$A$1:$F$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Methodology'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Methodology'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37680,7 +37680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -37702,65 +37702,77 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Archive scope</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Histogram, thematic coding, and frame analysis removed from the main dashboard.</t>
+          <t>Work in progress; the thematic and framing code and outputs have not been verified by a person.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Histogram</t>
+          <t>Archive scope</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Company-year six-term incidence per 100,000 extracted words; yearly statistics use population standard deviation.</t>
+          <t>Histogram, thematic coding, and frame analysis removed from the main dashboard.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Themes</t>
+          <t>Histogram</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Deterministic multi-label dictionary codes; one passage can receive multiple themes.</t>
+          <t>Company-year six-term incidence per 100,000 extracted words; yearly statistics use population standard deviation.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Frames</t>
+          <t>Themes</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Deterministic mutually exclusive primary frame assigned to each retained passage.</t>
+          <t>Deterministic multi-label dictionary codes; one passage can receive multiple themes.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Frames</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Deterministic mutually exclusive primary frame assigned to each retained passage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Exploratory coding only; independent human validation has not been completed.</t>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>No manual validation sample, inter-coder reliability study, or expert review has been completed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>